<commit_message>
Actualizar archivo de resultados.xlsx
</commit_message>
<xml_diff>
--- a/data/xlsx/resultados.xlsx
+++ b/data/xlsx/resultados.xlsx
@@ -5,16 +5,36 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FIERA\Desktop\AC\teamwork-ac-2025\data\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\menda\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89887B12-7508-4BD4-AB88-B0C40FCBEACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1D9965-5CEF-4C2E-901B-B72114AF577D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="16440" xr2:uid="{64E32888-7FF9-4962-B0B2-27FE6E737F4E}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{64E32888-7FF9-4962-B0B2-27FE6E737F4E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Hoja1!$A$2</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Hoja1!$A$3</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Hoja1!$B$3:$K$3</definedName>
+    <definedName name="_xlchart.v1.11" hidden="1">Hoja1!$B$4:$K$4</definedName>
+    <definedName name="_xlchart.v1.12" hidden="1">Hoja1!$A$2</definedName>
+    <definedName name="_xlchart.v1.13" hidden="1">Hoja1!$A$3</definedName>
+    <definedName name="_xlchart.v1.14" hidden="1">Hoja1!$A$4</definedName>
+    <definedName name="_xlchart.v1.15" hidden="1">Hoja1!$B$2:$K$2</definedName>
+    <definedName name="_xlchart.v1.16" hidden="1">Hoja1!$B$3:$K$3</definedName>
+    <definedName name="_xlchart.v1.17" hidden="1">Hoja1!$B$4:$K$4</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Hoja1!$A$4</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Hoja1!$B$2:$K$2</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Hoja1!$B$3:$K$3</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Hoja1!$B$4:$K$4</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Hoja1!$A$2</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Hoja1!$A$3</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Hoja1!$A$4</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Hoja1!$B$2:$K$2</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -252,7 +272,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -288,13 +308,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -310,6 +329,1903 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES"/>
+              <a:t>Tiempo</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-ES" baseline="0"/>
+              <a:t> medio de ejecución</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Hoja1!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SINGLE THREAD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Hoja1!$B$1:$R$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Hoja1!$L$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Media</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Hoja1!$B$2:$R$2</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Hoja1!$L$2</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>10.394</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-97A1-412B-8A66-0C467707654F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Hoja1!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>MULTI THREAD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Hoja1!$B$1:$R$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Hoja1!$L$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Media</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Hoja1!$B$3:$R$3</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Hoja1!$L$3</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6.588000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-97A1-412B-8A66-0C467707654F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Hoja1!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>SIMD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Hoja1!$B$1:$R$1</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Hoja1!$L$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Media</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Hoja1!$B$4:$R$4</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>Hoja1!$L$4</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>14.003</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-97A1-412B-8A66-0C467707654F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="317599520"/>
+        <c:axId val="317590880"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="317599520"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="317590880"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="317590880"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-ES"/>
+                  <a:t>Tiempo (s)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-ES"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="317599520"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:numDim type="val">
+        <cx:f dir="row">_xlchart.v1.3</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="1">
+      <cx:numDim type="val">
+        <cx:f dir="row">_xlchart.v1.4</cx:f>
+      </cx:numDim>
+    </cx:data>
+    <cx:data id="2">
+      <cx:numDim type="val">
+        <cx:f dir="row">_xlchart.v1.5</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Boxplot de tiempos de ejecución</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+            </a:rPr>
+            <a:t>Boxplot de tiempos de ejecución</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="boxWhisker" uniqueId="{BF91AD1F-C265-42D7-824F-590818849E31}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.0</cx:f>
+              <cx:v>SINGLE THREAD</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000004-851F-487B-BACA-778D4469B33A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.1</cx:f>
+              <cx:v>MULTI THREAD</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="1"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+        <cx:series layoutId="boxWhisker" uniqueId="{00000005-851F-487B-BACA-778D4469B33A}">
+          <cx:tx>
+            <cx:txData>
+              <cx:f>_xlchart.v1.2</cx:f>
+              <cx:v>SIMD</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:dataId val="2"/>
+          <cx:layoutPr>
+            <cx:statistics quartileMethod="exclusive"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="1"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling max="15" min="6"/>
+        <cx:title>
+          <cx:tx>
+            <cx:txData>
+              <cx:v>Tiempo (s)</cx:v>
+            </cx:txData>
+          </cx:tx>
+          <cx:txPr>
+            <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="es-ES" sz="900" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:sysClr>
+                  </a:solidFill>
+                  <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+                </a:rPr>
+                <a:t>Tiempo (s)</a:t>
+              </a:r>
+            </a:p>
+          </cx:txPr>
+        </cx:title>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+    <cx:legend pos="t" align="ctr" overlay="0"/>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="406">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>257174</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>167639</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>184784</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6CC2068E-FA9B-081C-23FA-558FCC4C4D6E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>372427</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>832486</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Gráfico 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A728E3A-3339-EB9F-A963-6D360C3257A1}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8708707" y="2667000"/>
+              <a:ext cx="4864419" cy="4762500"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-ES" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -629,7 +2545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C88A2E26-47F6-4350-B42D-F2D297B06200}">
-  <dimension ref="A1:S32"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
@@ -1020,12 +2936,10 @@
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="D14" s="1"/>
     </row>
-    <row r="32" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I32" s="15"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>